<commit_message>
feat: add security warning to printer section
</commit_message>
<xml_diff>
--- a/database.xlsx
+++ b/database.xlsx
@@ -2,8 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="2790" yWindow="2790" windowWidth="21600" windowHeight="11325" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="1. О Ферсол" sheetId="1" state="visible" r:id="rId1"/>
@@ -17,14 +18,14 @@
     <sheet name="9. Политики и заявления" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="162913" fullCalcOnLoad="1" refMode="R1C1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="17">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,112 +34,7 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <charset val="204"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <color theme="10"/>
-      <sz val="11"/>
-      <u val="single"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Montserrat Medium"/>
-      <color rgb="FF333E4C"/>
-      <sz val="13"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="14"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Montserrat Medium"/>
-      <color rgb="FF333E4C"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <name val="Montserrat Medium"/>
-      <color rgb="FF333E4C"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Times New Roman"/>
-      <charset val="204"/>
-      <family val="1"/>
-      <color theme="1"/>
-      <sz val="11.5"/>
-    </font>
-    <font>
-      <name val="Times New Roman"/>
-      <charset val="204"/>
-      <family val="1"/>
       <b val="1"/>
-      <color theme="1"/>
-      <sz val="11.5"/>
-    </font>
-    <font>
-      <name val="Times New Roman"/>
-      <charset val="204"/>
-      <family val="1"/>
-      <color rgb="FF000000"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <charset val="204"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color rgb="FF000000"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Times New Roman"/>
-      <charset val="204"/>
-      <family val="1"/>
-      <b val="1"/>
-      <color rgb="FF000000"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-      <color theme="1"/>
-      <sz val="11.5"/>
-    </font>
-    <font>
-      <name val="Times New Roman"/>
-      <charset val="204"/>
-      <family val="1"/>
-      <color theme="1"/>
-      <sz val="7"/>
-    </font>
-    <font>
-      <name val="Aptos"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Aptos"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color theme="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Aptos"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="12"/>
     </font>
   </fonts>
   <fills count="2">
@@ -149,7 +45,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -157,85 +53,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="7"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="5"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" indent="5"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="4"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="7"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="justify" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="justify" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -318,44 +155,44 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546A"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ED7D31"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="FFC000"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70AD47"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563C1"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954F72"/>
+        <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
@@ -382,15 +219,14 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
@@ -417,7 +253,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -429,142 +264,166 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="35000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="80000">
               <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="40000">
               <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
@@ -575,278 +434,361 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C43"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
-  <cols>
-    <col width="84.88671875" customWidth="1" style="4" min="2" max="2"/>
-    <col width="69.33203125" customWidth="1" style="4" min="3" max="3"/>
-  </cols>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" ht="50.4" customHeight="1" s="4">
-      <c r="A1" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>1.</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Fersol - провайдер индивидуальных проектных и консалтинговых решений в области сквозного управления технологическими процессами, обеспечения кадровым ресурсом и технической экспертизы</t>
         </is>
       </c>
-    </row>
-    <row r="2" s="4"/>
-    <row r="3" ht="50.4" customHeight="1" s="4">
-      <c r="B3" s="5" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
         <is>
           <t>Миссия Ферсол: мы соединяем передовые технологии с международной экспертизой для реализации сложных индустриальных проектов, запуска производств и создания инновационных продуктов</t>
         </is>
       </c>
-    </row>
-    <row r="6" ht="18" customHeight="1" s="4">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="C3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
         <is>
           <t>1.1.</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Ценности</t>
         </is>
       </c>
-      <c r="C6" s="2" t="n"/>
-    </row>
-    <row r="7" ht="18" customHeight="1" s="4">
-      <c r="A7" s="2" t="n"/>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="C6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
         <is>
           <t xml:space="preserve">ПРЕДПРИНИМАТЕЛЬСКИЙ ПОДХОД </t>
         </is>
       </c>
-      <c r="C7" s="2" t="n"/>
-    </row>
-    <row r="8" ht="98.40000000000001" customHeight="1" s="4">
-      <c r="A8" s="2" t="n"/>
-      <c r="B8" s="2" t="n"/>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
         <is>
           <t xml:space="preserve">Способность использовать текущую рыночную ситуацию в интересах компании, предлагая клиентам конкурентоспособные услуги премиального качества </t>
         </is>
       </c>
     </row>
-    <row r="9" ht="21.6" customHeight="1" s="4">
-      <c r="B9" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
         <is>
           <t>ЦЕЛОСТНОСТЬ</t>
         </is>
       </c>
-      <c r="C9" s="3" t="n"/>
-    </row>
-    <row r="10" ht="64.8" customHeight="1" s="4">
-      <c r="B10" s="2" t="n"/>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
         <is>
           <t>Честность, сплоченность, уважение и поддержание высоких моральных принципов как внутри организации, так и за её пределами</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="21.6" customHeight="1" s="4">
-      <c r="B11" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr"/>
+      <c r="B11" t="inlineStr">
         <is>
           <t>ОРИЕНТИРОВАННОСТЬ НА РЕЗУЛЬТАТ</t>
         </is>
       </c>
-      <c r="C11" s="3" t="n"/>
-    </row>
-    <row r="12" ht="86.40000000000001" customHeight="1" s="4">
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
         <is>
           <t>Четкая постановка целей, утверждение планов, контроль сроков исполнения, оценка результатов и постоянное стремление к совершенствованию</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="19.8" customHeight="1" s="4">
-      <c r="B13" s="1" t="inlineStr">
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" t="inlineStr">
         <is>
           <t>ВНИМАНИЕ К ЛЮДЯМ</t>
         </is>
       </c>
-    </row>
-    <row r="14" ht="86.40000000000001" customHeight="1" s="4">
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr"/>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr">
         <is>
           <t xml:space="preserve">Люди – основной капитал Fersol. Мы проявляем искреннее внимание и заботу о наших сотрудниках – как внутренних, так и контрактных. </t>
         </is>
       </c>
     </row>
-    <row r="17" ht="18" customHeight="1" s="4">
+    <row r="15">
+      <c r="A15" t="inlineStr"/>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr"/>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
+    </row>
+    <row r="17">
       <c r="A17" t="inlineStr">
         <is>
           <t>1.2.</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>Правила корпоративного внешнего вида</t>
         </is>
       </c>
-    </row>
-    <row r="18" ht="45" customHeight="1" s="4">
-      <c r="B18" s="6" t="inlineStr">
+      <c r="C17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
         <is>
           <t>Каждый работник Ферсол является ее представителем, у нас есть правила корпоративного внешнего вида, рекомендованные к соблюдению в течение рабочей недели.</t>
         </is>
       </c>
-    </row>
-    <row r="19" ht="15" customHeight="1" s="4">
-      <c r="B19" s="7" t="inlineStr">
+      <c r="C18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
         <is>
           <t>С понедельника по четверг</t>
         </is>
       </c>
-    </row>
-    <row r="20" ht="45" customHeight="1" s="4">
-      <c r="B20" s="6" t="inlineStr">
+      <c r="C19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
         <is>
           <t>Несмотря на то, что работники вправе иметь свободу самовыражения, офисным работникам рекомендуется выбирать одежду, обувь и аксессуары, соответствующие должности, должностным обязанностям и имиджу Компании.</t>
         </is>
       </c>
-    </row>
-    <row r="21" ht="75.59999999999999" customHeight="1" s="4">
-      <c r="B21" s="6" t="inlineStr">
+      <c r="C20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
         <is>
           <t>Стилем одежды работников Компании является приемлемое сочетание повседневного и делового стиля (Smart casual). Строго рекомендуется воздержаться от одежды, обуви, аксессуаров, которые могут быть отнесены к спортивному, небрежному, авангардному стилю. Одежда не должна быть вызывающей и откровенной. Рекомендованы спокойные тона одежды; желательно избегать ярких «кислотных» цветов.</t>
         </is>
       </c>
-    </row>
-    <row r="22" ht="26.4" customHeight="1" s="4">
-      <c r="B22" s="6" t="inlineStr">
+      <c r="C21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr"/>
+      <c r="B22" t="inlineStr">
         <is>
           <t xml:space="preserve">Для работников, у которых запланированы встречи с участием работников других организаций, рекомендован деловой стиль, подразумевающий деловой костюм или его эквивалент. </t>
         </is>
       </c>
-    </row>
-    <row r="23" ht="15" customHeight="1" s="4">
-      <c r="B23" s="7" t="inlineStr">
+      <c r="C22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr"/>
+      <c r="B23" t="inlineStr">
         <is>
           <t>Пятница</t>
         </is>
       </c>
-    </row>
-    <row r="24" ht="120" customHeight="1" s="4">
-      <c r="B24" s="6" t="inlineStr">
+      <c r="C23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr"/>
+      <c r="B24" t="inlineStr">
         <is>
           <t xml:space="preserve">В пятницу допускается менее формальный стиль одежды. Тем не менее рекомендуется придерживаться разумных рамок в связи с тем, что в этот день в офисе могут проводиться встречи с клиентами. Не допускается использование в одежде использование надписей или рисунков, которые потенциально могут быть расценены как оскорбление. Также рекомендовано воздержаться от использования во внешнем виде неформальных шортов, маек и другой одежды и обуви, предназначенных для отдыха, досуга или спорта. В пятницу разрешается ношение, свободной или спортивной одежды, если она изготовлена по заказу Компании или имеет символику Компании. </t>
         </is>
       </c>
-    </row>
-    <row r="25" ht="30" customHeight="1" s="4">
-      <c r="B25" s="6" t="inlineStr">
+      <c r="C24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr"/>
+      <c r="B25" t="inlineStr">
         <is>
           <t xml:space="preserve">Менее формальный стиль в пятницу для работников компании не является обязательным требованием. </t>
         </is>
       </c>
-    </row>
-    <row r="26" ht="39" customHeight="1" s="4">
-      <c r="B26" s="6" t="inlineStr">
+      <c r="C25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr"/>
+      <c r="B26" t="inlineStr">
         <is>
           <t>В случае если в пятницу у работников запланированы встречи с клиентами, менее формальный стиль одежды допускается только по предварительной договоренности с участниками встречи.</t>
         </is>
       </c>
-    </row>
-    <row r="27" ht="65.40000000000001" customHeight="1" s="4">
-      <c r="B27" s="6" t="inlineStr">
+      <c r="C26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr"/>
+      <c r="B27" t="inlineStr">
         <is>
           <t>Менее формальный стиль одежды в пятницу применим ко всем работникам организации за  исключением отдельных работников (отделов), для которых это может быть не применимо в силу объективных причин. Компания имеет право отменить менее формальный стиль одежды в пятницу на уровне всей организации и\или отдельного подразделения.</t>
         </is>
       </c>
-    </row>
-    <row r="28" ht="30" customHeight="1" s="4">
-      <c r="B28" s="6" t="inlineStr">
+      <c r="C27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr"/>
+      <c r="B28" t="inlineStr">
         <is>
           <t>Вопросы, связанные с корпоративным внешним видом, следует адресовать непосредственному руководителю или работникам отдела по работе с персоналом.</t>
         </is>
       </c>
-    </row>
-    <row r="30" ht="18" customHeight="1" s="4">
+      <c r="C28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr"/>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr"/>
+    </row>
+    <row r="30">
       <c r="A30" t="inlineStr">
         <is>
           <t>1.3.</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>Стандарты делового поведения Ферсол</t>
         </is>
       </c>
-    </row>
-    <row r="31" ht="105.6" customHeight="1" s="4">
-      <c r="B31" s="9" t="inlineStr">
+      <c r="C30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr"/>
+      <c r="B31" t="inlineStr">
         <is>
           <t xml:space="preserve">Политика в области этики: все работники Ферсол обязаны соблюдать все действующие законы, правила и нормативные акты, регулирующие их деятельность, и действовать добросовестно во всех отношениях при выполнении работ для Компании Ферсол. Работники должны надлежащим образом отражать фактическую информацию обо всей деятельности и сделках во всех записях, программах, отчетах, документах и учетных книгах, создаваемых в процессе работы или оказания услуг для Компании Ферсол. Эти сведения могут использоваться в качестве полной и достоверной информации в любых последующих записях и отчетах, составляемых Компанией Ферсол, или ее представителями в каких бы то ни было целях. </t>
         </is>
       </c>
-    </row>
-    <row r="32" ht="79.2" customHeight="1" s="4">
-      <c r="B32" s="9" t="inlineStr">
+      <c r="C31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr"/>
+      <c r="B32" t="inlineStr">
         <is>
           <t xml:space="preserve">Политика в отношении конфликта интересов: работники обязаны не допускать фактического наличия или возникновения конфликта между их собственными интересами и интересами Компании Ферсол. Например, Работники не вправе пользоваться возможностями, возникающими в процессе трудовой деятельности, и побуждать Компанию Ферсол или Клиента Работодателя оплачивать работникам работу, которая не была выполнена, либо работу, которая не была предусмотрена Работодателем и Клиентом. </t>
         </is>
       </c>
-    </row>
-    <row r="33" ht="79.2" customHeight="1" s="4">
-      <c r="B33" s="9" t="inlineStr">
+      <c r="C32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr"/>
+      <c r="B33" t="inlineStr">
         <is>
           <t>Политика в отношении конфликтов на рабочем месте: работники должны конструктивно взаимодействовать с другими отделами, решать возникающие вопросы в позитивном ключе, руководствуясь интересами компании (а не собственного отдела/должности). Работники не должны допускать внутренние конфликты, споры и розни между отделами или сотрудниками. Работники не должны допускать любые конфликты интересов, личные конфликты, неприязни, недружественные и неконструктивные действия по отношению к коллегам и компании Ферсол.</t>
         </is>
       </c>
-    </row>
-    <row r="34" ht="79.2" customHeight="1" s="4">
-      <c r="B34" s="9" t="inlineStr">
+      <c r="C33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr"/>
+      <c r="B34" t="inlineStr">
         <is>
           <t>Политика в отношении корпоративного имущества: работники обязаны сохранять имущество своего Работодателя, если использование такого имущества работниками предусмотрено для осуществления трудовой деятельности, они должны использовать его эффективным образом в интересах Работодателя. Запрещается использование имущества Работодателя Работником в личных целях. Имущество Работодателя состоит из физического (осязаемого) и неосязаемого имущества (интеллектуальной собственности), включающего конфиденциальную информацию Компании Ферсол.</t>
         </is>
       </c>
-    </row>
-    <row r="35" ht="39.6" customHeight="1" s="4">
-      <c r="B35" s="8" t="inlineStr">
+      <c r="C34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr"/>
+      <c r="B35" t="inlineStr">
         <is>
           <t>Работники не вправе без соответствующего разрешения использовать и разглашать в то или иное время в процессе и после трудоустройства конфиденциальную информацию, полученную из любого источника в ходе осуществления трудовой деятельности.</t>
         </is>
       </c>
-    </row>
-    <row r="36" ht="39.6" customHeight="1" s="4">
-      <c r="B36" s="8" t="inlineStr">
+      <c r="C35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr"/>
+      <c r="B36" t="inlineStr">
         <is>
           <t>Конфиденциальной информацией считается вся закрытая информация о договорах компании Ферсол, планах, открытиях, доходах, конкурсных заявках, технологиях, рабочих процессах и персонале Компании Ферсол и ее Клиентов.</t>
         </is>
       </c>
-    </row>
-    <row r="37" ht="79.2" customHeight="1" s="4">
-      <c r="B37" s="9" t="inlineStr">
+      <c r="C36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr"/>
+      <c r="B37" t="inlineStr">
         <is>
           <t xml:space="preserve">Политика в отношении подарков и развлечений: если работникам предлагаются подарки либо нестандартные, чрезмерные, дорогостоящие или необычные развлечения в связи с услугами, оказываемыми Компанией Ферсол Клиенту по договору(ам), работники должны поставить в известность о таких подарках либо приглашениях принять участие в нестандартных, чрезмерных, дорогостоящих и необычных развлечениях Компанию Ферсол: непосредственного руководителя и службу персонала. </t>
         </is>
       </c>
-    </row>
-    <row r="38" ht="92.40000000000001" customHeight="1" s="4">
-      <c r="B38" s="10" t="inlineStr">
+      <c r="C37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr"/>
+      <c r="B38" t="inlineStr">
         <is>
           <t>Политика в отношении занятия должности директора других организаций: работники не могут занимать должности директоров неаффилированных коммерческих организаций и не вправе принимать новые назначения на должность директора, которые могут повлечь за собой возникновение конфликта интересов либо помешать исполнению обязательств Компании Ферсол перед Клиентом. Сведения о любых занимаемых должностях, которые потенциально могут привести к возникновению конфликта интересов, должны доводиться до сведения Компании Ферсол до того, как Работник будет допущен к работе.</t>
         </is>
       </c>
-    </row>
-    <row r="39" ht="18" customHeight="1" s="4">
+      <c r="C38" t="inlineStr"/>
+    </row>
+    <row r="39">
       <c r="A39" t="inlineStr">
         <is>
           <t>1.4.</t>
         </is>
       </c>
-      <c r="B39" s="2" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>Соцсети</t>
         </is>
       </c>
+      <c r="C39" t="inlineStr"/>
     </row>
     <row r="40">
+      <c r="A40" t="inlineStr"/>
       <c r="B40" t="inlineStr">
         <is>
           <t>корпоративный чат WhatsApp</t>
@@ -859,6 +801,7 @@
       </c>
     </row>
     <row r="41">
+      <c r="A41" t="inlineStr"/>
       <c r="B41" t="inlineStr">
         <is>
           <t>TG-канал</t>
@@ -871,6 +814,7 @@
       </c>
     </row>
     <row r="42">
+      <c r="A42" t="inlineStr"/>
       <c r="B42" t="inlineStr">
         <is>
           <t>ВК</t>
@@ -882,96 +826,92 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="18" customHeight="1" s="4">
+    <row r="43">
       <c r="A43" t="inlineStr">
         <is>
           <t>1.5.</t>
         </is>
       </c>
-      <c r="B43" s="2" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t xml:space="preserve">Список контактов </t>
         </is>
       </c>
-      <c r="C43" s="11" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>U:\Public\HR docs for employees\Phone list.xlsx</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId1"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="FFFFFF00"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
-  <cols>
-    <col width="58.6640625" customWidth="1" style="4" min="2" max="2"/>
-  </cols>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" ht="18" customHeight="1" s="4">
-      <c r="A1" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>2.1.</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Даты выплаты</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="105" customHeight="1" s="4">
-      <c r="B2" s="12" t="inlineStr">
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+      <c r="B2" t="inlineStr">
         <is>
           <t>Оплата труда работников производится в соответствии с требованиями законодательства РФ. Выплата заработной платы Работникам производится не реже, чем два раза в месяц в соответствии с утвержденным Работодателем Графиком выплаты заработной платы. Первая часть выплачивается 25 числа текущего месяца, полный расчет производится 10 числа следующего месяца.</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="18" customHeight="1" s="4">
+    <row r="3">
       <c r="A3" t="inlineStr">
         <is>
           <t>2.2.</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Реквизиты и зарплатный проект</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="60" customHeight="1" s="4">
-      <c r="B4" s="12" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
         <is>
           <t>Заработная плата выплачивается Работнику путем перевода денежных средств на банковский счет Работника как в рамках зарплатного проекта Работодателя, так и на любой другой счет Работника по его желанию.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" s="4">
+    <row r="5">
       <c r="A5" t="inlineStr">
         <is>
           <t>2.3.</t>
         </is>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Порядок оплаты труда работников</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="180" customHeight="1" s="4">
-      <c r="B6" s="15" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
         <is>
           <t>Должностной оклад (месячная тарифная ставка) начисляется работнику полностью, если фактически отработанное время равно норме рабочего времени (в рабочих днях), установленной производственным календарем на соответствующий месяц.              
 При отклонении фактически отработанного времени от нормы, должностной оклад начисляется за фактически отработанное время исходя из дневной тарифной ставки.
@@ -980,7 +920,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -991,96 +931,99 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
-  <cols>
-    <col width="72.21875" customWidth="1" style="4" min="2" max="2"/>
-  </cols>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" ht="18" customHeight="1" s="4">
-      <c r="A1" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>3.</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Испытательный срок</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="54.6" customHeight="1" s="4">
+    <row r="2">
       <c r="A2" t="inlineStr">
         <is>
           <t>3.1.</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Цель испытательного срока - проверка соответствия работника поручаемой ему деятельности непосредственно в рабочей обстановке.</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="30" customHeight="1" s="4">
-      <c r="B3" s="6" t="inlineStr">
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
         <is>
           <t>Продолжительность испытательного срока указывается в трудовом договоре и в приказе о приеме на работу.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="60" customHeight="1" s="4">
-      <c r="B4" s="6" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
         <is>
           <t>В испытательный срок не засчитывается период временной нетрудоспособности, отпуска и другие периоды, когда работник фактически отсутствовал на работе. При наличии периодов отсутствия испытательный срок продлевается на тот же период.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="60" customHeight="1" s="4">
-      <c r="B5" s="6" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+      <c r="B5" t="inlineStr">
         <is>
           <t>При неудовлетворительном результате испытания работодатель имеет право до истечения срока испытания расторгнуть трудовой договор с работником, предупредив его об этом в письменном виде не позднее чем за три дня.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="30" customHeight="1" s="4">
-      <c r="B6" s="6" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
         <is>
           <t>При неудовлетворительном результате испытания расторжение трудового договора работника производится без выплаты выходного пособия.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="45" customHeight="1" s="4">
-      <c r="B7" s="6" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
         <is>
           <t>Если испытательный срок истек, а сотрудник продолжает работать, он считается выдержавшим испытание. Последующее расторжение трудового договора допускается только на общих основаниях.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="60" customHeight="1" s="4">
-      <c r="B8" s="6" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" t="inlineStr">
         <is>
           <t>Если в период испытания работник придет к выводу, что предложенная ему работа не является для него подходящей, то он имеет право расторгнуть трудовой договор по собственному желанию, предупредив об этом работодателя в письменной форме за три дня.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="18" customHeight="1" s="4">
+    <row r="9">
       <c r="A9" t="inlineStr">
         <is>
           <t>3.2.</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>Порядок работы на испытательном сроке</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="237" customHeight="1" s="4">
+    <row r="10">
       <c r="A10" t="inlineStr">
         <is>
           <t>3.2.</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t xml:space="preserve">Руководитель с вновь принятым сотрудником (в течение первой недели после зачисления) составляют устный или письменный план работы на время испытательного срока, который включает в себя задания и сроки их выполнения. 
 В течение испытательного срока руководитель или куратор поручает задания работнику. Задания могут быть переданы как устно, так и письменно, в том числе по электронной почте.
@@ -1091,7 +1034,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -1102,54 +1045,55 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
-  <cols>
-    <col width="12" customWidth="1" style="4" min="1" max="1"/>
-    <col width="87.77734375" customWidth="1" style="4" min="2" max="2"/>
-  </cols>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 0</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>ДМС</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="18" customHeight="1" s="4">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="2">
+      <c r="A2" t="inlineStr">
         <is>
           <t>4.1.</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Порядок оформления ДМС</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="56.4" customHeight="1" s="4">
-      <c r="A3" s="17" t="n"/>
-      <c r="B3" s="6" t="inlineStr">
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
         <is>
           <t>Добровольное медицинское страхование «Согаз» в месте постоянного проживания после трех месяцев работы в Ферсол. Менеджер по персоналу подает заявку на прикрепление к договору со страховой компанией. Полис ДМС приложения к нему приходит на личный email работника.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="56.4" customHeight="1" s="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>4.2.</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Объем услуг</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="259.2" customHeight="1" s="4">
-      <c r="A5" s="17" t="n"/>
-      <c r="B5" s="14" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+      <c r="B5" t="inlineStr">
         <is>
           <t>Чтобы получать услуги по Вашему полису:
 1. Скачайте мобильное приложение «СОГАЗ – здоровье и страхование» по ссылке https://www.sogaz.ru/m 
@@ -1169,46 +1113,48 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="18" customHeight="1" s="4">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="inlineStr">
         <is>
           <t>4.3.</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Прикрепление родственников</t>
         </is>
       </c>
     </row>
     <row r="7">
+      <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
           <t>Прикрепление родственников возможно по согласованию с менеджером по персоналу на услувиях ежемесячного удержания стоимости ДМС из зарплаты работника.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="24" customHeight="1" s="4">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t xml:space="preserve">4.4. </t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>Полис путешественника</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="60" customHeight="1" s="4">
-      <c r="B9" s="6" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
         <is>
           <t xml:space="preserve">Оформление полиса страхование путешествующих «Согаз» с покрытием $35000 возможно после трех месяцев работы в Ферсол. Полис оформляется по необходимости и привязан к сроку действия полиса ДМС. Для оформления нужно направить копию загранпаспорта менеджеру по персоналу. </t>
         </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -1218,42 +1164,43 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
-  <cols>
-    <col width="10.6640625" customWidth="1" style="4" min="1" max="1"/>
-    <col width="9" customWidth="1" style="4" min="2" max="2"/>
-    <col width="76.6640625" customWidth="1" style="4" min="3" max="3"/>
-  </cols>
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" ht="18" customHeight="1" s="4">
-      <c r="A1" s="18" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>5.</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Отпуск и больничный</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="18" customHeight="1" s="4">
-      <c r="A2" s="13" t="n"/>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
           <t>5.1.</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Когда можно взять отпуск?</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="231" customHeight="1" s="4">
-      <c r="A3" s="13" t="n"/>
-      <c r="C3" s="23" t="inlineStr">
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
         <is>
           <t>Право на использование отпуска за первый год работы возникает у работника по истечении шести месяцев его непрерывной работы у данного работодателя. По договоренности с руководителем оплачиваемый отпуск работнику может быть предоставлен и до истечения шести месяцев. 
 Продолжительность ежегодного оплачиваемого отпуска для работников составляет двадцать восемь календарных дней, если иное не предусмотрено законодательством. Допускается разделение отпуска на части при условии, что одна из частей отпуска должна составлять не менее 14 календарных дней.
@@ -1261,80 +1208,84 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="18" customHeight="1" s="4">
-      <c r="A4" s="13" t="n"/>
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
           <t>5.2.</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>За какое время подать заявление?</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="30" customHeight="1" s="4">
-      <c r="A5" s="13" t="n"/>
-      <c r="C5" s="22" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
         <is>
           <t>Заявление на оплачиваемый отпуск нужно подать не позднее, чем за 5 рабочих дней до его начала.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="18" customHeight="1" s="4">
-      <c r="A6" s="13" t="n"/>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
           <t>5.3.</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Почему я получил меньше из-за отпуска?</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="90" customHeight="1" s="4">
-      <c r="A7" s="13" t="n"/>
-      <c r="C7" s="23" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
         <is>
           <t>Такое возможно, так как отпуск рассчитывается исходя из среднего заработка в календарных днях. Грубо оплату одного дня отпуска можно посчитать так: средний заработок за месяц/29,3. 
 Чтобы нивелировать разницу можно добавить выходные дни к периоду отпуска, они тоже будут оплачены.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="18" customHeight="1" s="4">
-      <c r="A8" s="13" t="n"/>
+    <row r="8">
+      <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
           <t>5.4.</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Отпуск без сохранения зп</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="n"/>
-    </row>
-    <row r="10" ht="18" customHeight="1" s="4">
-      <c r="A10" s="13" t="n"/>
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
           <t>5.5.</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>Заявления на отпуск оплачиваемый и неоплачиваемый</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="21" t="n"/>
+      <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
           <t>ЧАЗ</t>
@@ -1347,7 +1298,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="21" t="n"/>
+      <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
           <t xml:space="preserve"> Сервис</t>
@@ -1359,41 +1310,45 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="18" customHeight="1" s="4">
-      <c r="B13" s="19" t="inlineStr">
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" t="inlineStr">
         <is>
           <t xml:space="preserve">5.6. </t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>Когда придут отпускные</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="45" customHeight="1" s="4">
-      <c r="B14" s="19" t="n"/>
-      <c r="C14" s="23" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="inlineStr"/>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr">
         <is>
           <t>Оплата отпуска будет начислена за 3 календарных дня до начала отпуска. Если вы не получили оплату, обратитесь к менеджеру по персоналу.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="18" customHeight="1" s="4">
-      <c r="A15" s="19" t="n"/>
+    <row r="15">
+      <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
           <t>5.7.</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>Больничный</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="61.8" customHeight="1" s="4">
-      <c r="C16" s="23" t="inlineStr">
+    <row r="16">
+      <c r="A16" t="inlineStr"/>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr">
         <is>
           <t xml:space="preserve">Больничный лист оформляется в электронном виде — самостоятельно приносить документы работодателю или отправлять их в фонд не нужно. 
 Если вам был открыт больничный - сообщите об этом руководителю и менеджеру по персоналу.
@@ -1401,21 +1356,17 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="30" customHeight="1" s="4">
-      <c r="C17" s="23" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr"/>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr">
         <is>
           <t xml:space="preserve">Работникам, прошедшим испытательный срок, производится доплата до фактического заработка за первые 14 дней в год. </t>
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1" s="4">
-      <c r="C18" s="23" t="n"/>
-    </row>
-    <row r="24">
-      <c r="C24" s="24" t="n"/>
-    </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -1425,67 +1376,147 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
-  <cols>
-    <col width="48.6640625" customWidth="1" style="4" min="2" max="2"/>
-  </cols>
+  <dimension ref="A1:B22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" ht="18" customHeight="1" s="4">
-      <c r="B1" s="2" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 0</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>6. Печать документов</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="18" customHeight="1" s="4">
+    <row r="2">
       <c r="A2" t="inlineStr">
         <is>
           <t>6.1.</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Код к принтеру</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="73.2" customHeight="1" s="4">
-      <c r="B3" s="23" t="inlineStr">
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
         <is>
           <t>Доступ к принтеру возможен по индивидуальному номеру ID для печати/копирования, который пришел вам на email от canon@fersol.org. Если такого кода не поступило - обратитесь к IT-специалисту</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="23.4" customHeight="1" s="4">
+    <row r="4">
       <c r="A4" t="inlineStr">
         <is>
           <t>6.2.</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Выбор принтера</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="30" customHeight="1" s="4">
-      <c r="B5" s="23" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+      <c r="B5" t="inlineStr">
         <is>
           <t>При отправке документов на печать выбирайте принтер Fersol_printer на srv-prn:</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="30" customHeight="1" s="4">
-      <c r="B20" s="23" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr"/>
+      <c r="B11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+      <c r="B12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr"/>
+      <c r="B14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr"/>
+      <c r="B15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr"/>
+      <c r="B16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr"/>
+      <c r="B17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+      <c r="B18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr"/>
+      <c r="B19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
         <is>
           <t>Для форматирования файла в формат PDF и его сохранения выбирайте принтер PDF24</t>
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>6.3.</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Безопасность</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr"/>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>В целях безопасности нельзя оставлять документы на принтере!</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" paperSize="9"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -1496,18 +1527,15 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
-  <cols>
-    <col width="51.33203125" customWidth="1" style="4" min="2" max="2"/>
-  </cols>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" ht="18" customHeight="1" s="4">
-      <c r="A1" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>7.</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Удаленный доступ </t>
         </is>
@@ -1525,76 +1553,83 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="45" customHeight="1" s="4">
-      <c r="B3" s="20" t="inlineStr">
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
         <is>
           <t>Для удаленного доступа к рабочему столу в интернет-браузере используем ссылку fersol.cloud.mts.ru/logon/LogonPoint/index.html</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="30" customHeight="1" s="4">
-      <c r="B4" s="20" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
         <is>
           <t>В первый раз предложит скачать Citrix - программу для подключения.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="18" customHeight="1" s="4">
+    <row r="5">
       <c r="A5" t="inlineStr">
         <is>
           <t>7.2.</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t xml:space="preserve"> Манго-телефония</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="111.6" customHeight="1" s="4">
-      <c r="B6" s="20" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
         <is>
           <t xml:space="preserve"> В обязательном порядке установить на телефон (рабочий или личный) приложение Mango Talker, это заменит стационарный телефон в полной мере (поддерживаются Android, iOS и Huawei) 
 Авторизация в приложении – вводите свой рабочий почтовый ящик, на почту получаете код, вводите его в приложении.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="45" customHeight="1" s="4">
-      <c r="B7" s="6" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
         <is>
           <t xml:space="preserve"> Для работы приложения необходим лишь интернет. Все настройки уже сделаны – необходимо лишь залогиниться.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="30" customHeight="1" s="4">
-      <c r="B8" s="6" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" t="inlineStr">
         <is>
           <t>Приложение работает только на территории России, звонки доступны по миру</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="60" customHeight="1" s="4">
-      <c r="B9" s="20" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
         <is>
           <t xml:space="preserve"> Более подробная информация размещена здесь 
 https://www.mango-office.ru/support/virtualnaya_ats/rukovodstvo_polzovatelya/rukovodstvo_polzovatelya_mango_talker/</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="18" customHeight="1" s="4">
+    <row r="10">
       <c r="A10" t="inlineStr">
         <is>
           <t>7.3.</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>Офис 365</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="43.2" customHeight="1" s="4">
-      <c r="B11" s="14" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr"/>
+      <c r="B11" t="inlineStr">
         <is>
           <t>Доступа к почте в браузере с мобильный устройств возможен по ссылке
 https://m365.cloud.microsoft/</t>
@@ -1602,7 +1637,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -1612,30 +1647,42 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:D12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
-  <cols>
-    <col width="3" customWidth="1" style="4" min="2" max="2"/>
-    <col width="22" customWidth="1" style="4" min="4" max="4"/>
-  </cols>
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" ht="18" customHeight="1" s="4">
-      <c r="B1" s="16" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 0</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>8.      Как закрыть офис</t>
         </is>
       </c>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 2</t>
+        </is>
+      </c>
     </row>
     <row r="2">
+      <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
           <t>Вот алгоритм действий, если вы закрываете двери офиса в конце рабочего дня.</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr"/>
     </row>
     <row r="4">
+      <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
           <t>1.</t>
@@ -1648,6 +1695,7 @@
       </c>
     </row>
     <row r="5">
+      <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
           <t>2.</t>
@@ -1660,6 +1708,7 @@
       </c>
     </row>
     <row r="6">
+      <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
           <t>3.</t>
@@ -1672,6 +1721,7 @@
       </c>
     </row>
     <row r="7">
+      <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
           <t>4.</t>
@@ -1684,13 +1734,16 @@
       </c>
     </row>
     <row r="8">
+      <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
           <t>Затем, убрать печать в пластиковый кармашек, просунуть в щель под дверь 429</t>
         </is>
       </c>
+      <c r="C8" t="inlineStr"/>
     </row>
     <row r="9">
+      <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
           <t>5.</t>
@@ -1702,22 +1755,31 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
+    </row>
     <row r="11">
+      <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
           <t xml:space="preserve">Помните, что на дверях 2 замка – электронный и механический. Если вы остаетесь одни в офисе, не забывайте о пропуске. </t>
         </is>
       </c>
+      <c r="C11" t="inlineStr"/>
     </row>
     <row r="12">
+      <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
           <t>В случае, если вы оставили пропуск в офисе и некому открыть дверь, пишите в общий чат Fersol.</t>
         </is>
       </c>
+      <c r="C12" t="inlineStr"/>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -1727,9 +1789,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:C6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 0</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 1</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 2</t>
+        </is>
+      </c>
+    </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
@@ -1741,13 +1820,16 @@
           <t>Все политики компании расположены по ссылке:</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr"/>
     </row>
     <row r="3">
+      <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
           <t>U:\Public\HR docs for employees\Internal Policies\Ферсол</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1760,8 +1842,10 @@
           <t>Формы заявлений</t>
         </is>
       </c>
+      <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
+      <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
           <t>Сервис:</t>
@@ -1774,6 +1858,7 @@
       </c>
     </row>
     <row r="6">
+      <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
           <t>ЧАЗ:</t>
@@ -1786,6 +1871,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: rename sub-companies to Fersol Service and Fersol CHAZ
</commit_message>
<xml_diff>
--- a/database.xlsx
+++ b/database.xlsx
@@ -1288,7 +1288,7 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ЧАЗ</t>
+          <t>Ферсол ЧАЗ</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1848,7 +1848,7 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Сервис:</t>
+          <t>Ферсол Сервис</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1861,7 +1861,7 @@
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ЧАЗ:</t>
+          <t>Ферсол ЧАЗ</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">

</xml_diff>

<commit_message>
feat: replace WhatsApp link with Telegram link
</commit_message>
<xml_diff>
--- a/database.xlsx
+++ b/database.xlsx
@@ -791,12 +791,12 @@
       <c r="A40" t="inlineStr"/>
       <c r="B40" t="inlineStr">
         <is>
-          <t>корпоративный чат WhatsApp</t>
+          <t>корпоративный чат Telegram</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>https://chat.whatsapp.com/FOygbIFvlNG1IAq2xSGPRf</t>
+          <t>https://t.me/+A8pvP2lWQs5mOGEy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add telegram link to 'close office' section
</commit_message>
<xml_diff>
--- a/database.xlsx
+++ b/database.xlsx
@@ -1773,10 +1773,14 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>В случае, если вы оставили пропуск в офисе и некому открыть дверь, пишите в общий чат Fersol.</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr"/>
+          <t>В случае, если вы оставили пропуск в офисе и некому открыть дверь, пишите в общий чат Fersol</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>https://t.me/+A8pvP2lWQs5mOGEy</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>